<commit_message>
Subida inicial del recomendador inteligente de Sabaneta
</commit_message>
<xml_diff>
--- a/recomendador_sabaneta/data/base_actualizada.xlsx
+++ b/recomendador_sabaneta/data/base_actualizada.xlsx
@@ -37,14 +37,14 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhzufvoaGk4DuuCXa87oo9Z+Fm/zw=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mig0PM/i++D6oLh/q/dfvryoRjZGw=="/>
     </ext>
   </extLst>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1157" uniqueCount="405">
   <si>
     <t>Introducción teorica sobre el ciclo de vida de proyecto de ML</t>
   </si>
@@ -1120,6 +1120,132 @@
     <t>Calle 72 Sur # 44-05</t>
   </si>
   <si>
+    <t>La Colmena sur</t>
+  </si>
+  <si>
+    <t>Ferretero</t>
+  </si>
+  <si>
+    <t>Todo en llaves de seguridad</t>
+  </si>
+  <si>
+    <t>Carrera 45 # 72 Sur-35</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/cafemilagrooficial/</t>
+  </si>
+  <si>
+    <t>Jvan Londoño</t>
+  </si>
+  <si>
+    <t>Publicitario</t>
+  </si>
+  <si>
+    <t>Fotografía</t>
+  </si>
+  <si>
+    <t>Fotografía, retratos, publicidad</t>
+  </si>
+  <si>
+    <t>Calle 72 Sur #45 A-60</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/jvan.londono.studio/</t>
+  </si>
+  <si>
+    <t>Guillego Estudio Fotográfico</t>
+  </si>
+  <si>
+    <t>Servicio fotografico, eventos sociales, diseño e impresión</t>
+  </si>
+  <si>
+    <t>Calle 72 Sur # 45 A -09</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/gestudiofotografico/?hl=es</t>
+  </si>
+  <si>
+    <t>La Vaca Lola</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>Comercio Minorista</t>
+  </si>
+  <si>
+    <t>Productos para bebe</t>
+  </si>
+  <si>
+    <t>Carrera 47 # 75 Sur 16</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/p/La-vaca-Lola-Tienda-para-Pekes-100062939305948/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/lavacalolatiendaparapekes/?hl=es-la</t>
+  </si>
+  <si>
+    <t>Rocky Cueros</t>
+  </si>
+  <si>
+    <t>Venta accesorios para montar caballo, monturas, alfombras,frenos, riendas, aperos</t>
+  </si>
+  <si>
+    <t>Calle 72 Sur # 45A-10</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/rockycueross/?locale=es_LA</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/rockycueros/</t>
+  </si>
+  <si>
+    <t>Sastreria DYD</t>
+  </si>
+  <si>
+    <t>Calle 69 Sur # 46-27</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/sastrw/?locale=es_LA</t>
+  </si>
+  <si>
+    <t>Colombia	Antioquia	Sabaneta</t>
+  </si>
+  <si>
+    <t>Empeliculados</t>
+  </si>
+  <si>
+    <t>Tienda de articulos de colección</t>
+  </si>
+  <si>
+    <t>Carrera 48 # 76D Sur 52</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/empeliculadoscol/</t>
+  </si>
+  <si>
+    <t>Tienda de Regalos Sabaneta</t>
+  </si>
+  <si>
+    <t>Anchetas, desayunos sorpresa, empaques para regalo, cajas y accesorios</t>
+  </si>
+  <si>
+    <t>Calle 72 Sur #46-37</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/tiendaderegalossabaneta/?hl=es</t>
+  </si>
+  <si>
+    <t>Proyecto y Enfoque Inmobiliario</t>
+  </si>
+  <si>
+    <t>Cl 66 S # 43C-84</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/p/Proyecto-Y-Enfoque-Inmobiliario-100083624130170/</t>
+  </si>
+  <si>
     <t>MV</t>
   </si>
   <si>
@@ -1139,7 +1265,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -1190,6 +1316,12 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1205,7 +1337,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1234,6 +1366,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -14249,18 +14384,42 @@
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="1"/>
-      <c r="B93" s="1"/>
-      <c r="C93" s="1"/>
-      <c r="D93" s="1"/>
-      <c r="E93" s="1"/>
-      <c r="F93" s="1"/>
-      <c r="G93" s="1"/>
-      <c r="H93" s="1"/>
-      <c r="I93" s="1"/>
-      <c r="J93" s="1"/>
-      <c r="K93" s="1"/>
-      <c r="L93" s="1"/>
-      <c r="M93" s="1"/>
+      <c r="B93" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="D93" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="E93" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G93" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H93" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I93" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="J93" s="8">
+        <v>3.155434962E9</v>
+      </c>
+      <c r="K93" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L93" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="M93" s="12" t="s">
+        <v>362</v>
+      </c>
       <c r="N93" s="1"/>
       <c r="O93" s="1"/>
       <c r="P93" s="1"/>
@@ -14275,18 +14434,42 @@
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="1"/>
-      <c r="B94" s="1"/>
-      <c r="C94" s="1"/>
-      <c r="D94" s="1"/>
-      <c r="E94" s="1"/>
-      <c r="F94" s="1"/>
-      <c r="G94" s="1"/>
-      <c r="H94" s="1"/>
-      <c r="I94" s="1"/>
-      <c r="J94" s="1"/>
-      <c r="K94" s="1"/>
-      <c r="L94" s="1"/>
-      <c r="M94" s="1"/>
+      <c r="B94" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="E94" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="F94" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G94" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H94" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I94" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="J94" s="8">
+        <v>3.218714789E9</v>
+      </c>
+      <c r="K94" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L94" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="M94" s="10" t="s">
+        <v>368</v>
+      </c>
       <c r="N94" s="1"/>
       <c r="O94" s="1"/>
       <c r="P94" s="1"/>
@@ -14301,18 +14484,42 @@
     </row>
     <row r="95" ht="14.25" customHeight="1">
       <c r="A95" s="1"/>
-      <c r="B95" s="1"/>
-      <c r="C95" s="1"/>
-      <c r="D95" s="1"/>
-      <c r="E95" s="1"/>
-      <c r="F95" s="1"/>
-      <c r="G95" s="1"/>
-      <c r="H95" s="1"/>
-      <c r="I95" s="1"/>
-      <c r="J95" s="1"/>
-      <c r="K95" s="1"/>
-      <c r="L95" s="1"/>
-      <c r="M95" s="1"/>
+      <c r="B95" s="8" t="s">
+        <v>369</v>
+      </c>
+      <c r="C95" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="D95" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="E95" s="8" t="s">
+        <v>370</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H95" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I95" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="J95" s="8">
+        <v>3.218054649E9</v>
+      </c>
+      <c r="K95" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L95" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="M95" s="12" t="s">
+        <v>372</v>
+      </c>
       <c r="N95" s="1"/>
       <c r="O95" s="1"/>
       <c r="P95" s="1"/>
@@ -14327,18 +14534,42 @@
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="1"/>
-      <c r="B96" s="1"/>
-      <c r="C96" s="1"/>
-      <c r="D96" s="1"/>
-      <c r="E96" s="1"/>
-      <c r="F96" s="1"/>
-      <c r="G96" s="1"/>
-      <c r="H96" s="1"/>
-      <c r="I96" s="1"/>
-      <c r="J96" s="1"/>
-      <c r="K96" s="1"/>
-      <c r="L96" s="1"/>
-      <c r="M96" s="1"/>
+      <c r="B96" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D96" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="E96" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I96" s="8" t="s">
+        <v>377</v>
+      </c>
+      <c r="J96" s="8">
+        <v>3.006760642E9</v>
+      </c>
+      <c r="K96" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L96" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="M96" s="11" t="s">
+        <v>379</v>
+      </c>
       <c r="N96" s="1"/>
       <c r="O96" s="1"/>
       <c r="P96" s="1"/>
@@ -14353,18 +14584,42 @@
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="1"/>
-      <c r="B97" s="1"/>
-      <c r="C97" s="1"/>
-      <c r="D97" s="1"/>
-      <c r="E97" s="1"/>
-      <c r="F97" s="1"/>
-      <c r="G97" s="1"/>
-      <c r="H97" s="1"/>
-      <c r="I97" s="1"/>
-      <c r="J97" s="1"/>
-      <c r="K97" s="1"/>
-      <c r="L97" s="1"/>
-      <c r="M97" s="1"/>
+      <c r="B97" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="C97" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D97" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="E97" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G97" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H97" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I97" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="J97" s="8">
+        <v>3.217511266E9</v>
+      </c>
+      <c r="K97" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L97" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="M97" s="10" t="s">
+        <v>384</v>
+      </c>
       <c r="N97" s="1"/>
       <c r="O97" s="1"/>
       <c r="P97" s="1"/>
@@ -14379,18 +14634,42 @@
     </row>
     <row r="98" ht="14.25" customHeight="1">
       <c r="A98" s="1"/>
-      <c r="B98" s="1"/>
-      <c r="C98" s="1"/>
-      <c r="D98" s="1"/>
-      <c r="E98" s="1"/>
-      <c r="F98" s="1"/>
-      <c r="G98" s="1"/>
-      <c r="H98" s="1"/>
-      <c r="I98" s="1"/>
-      <c r="J98" s="1"/>
-      <c r="K98" s="1"/>
-      <c r="L98" s="1"/>
-      <c r="M98" s="1"/>
+      <c r="B98" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="D98" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="E98" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H98" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I98" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="J98" s="8">
+        <v>3.152775314E9</v>
+      </c>
+      <c r="K98" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L98" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="M98" s="8" t="s">
+        <v>388</v>
+      </c>
       <c r="N98" s="1"/>
       <c r="O98" s="1"/>
       <c r="P98" s="1"/>
@@ -14405,18 +14684,42 @@
     </row>
     <row r="99" ht="14.25" customHeight="1">
       <c r="A99" s="1"/>
-      <c r="B99" s="1"/>
-      <c r="C99" s="1"/>
-      <c r="D99" s="1"/>
-      <c r="E99" s="1"/>
-      <c r="F99" s="1"/>
-      <c r="G99" s="1"/>
-      <c r="H99" s="1"/>
-      <c r="I99" s="1"/>
-      <c r="J99" s="1"/>
-      <c r="K99" s="1"/>
-      <c r="L99" s="1"/>
-      <c r="M99" s="1"/>
+      <c r="B99" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="C99" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D99" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="E99" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G99" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H99" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I99" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="J99" s="8">
+        <v>3.21749353E9</v>
+      </c>
+      <c r="K99" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L99" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="M99" s="11" t="s">
+        <v>392</v>
+      </c>
       <c r="N99" s="1"/>
       <c r="O99" s="1"/>
       <c r="P99" s="1"/>
@@ -14431,18 +14734,42 @@
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="1"/>
-      <c r="B100" s="1"/>
-      <c r="C100" s="1"/>
-      <c r="D100" s="1"/>
-      <c r="E100" s="1"/>
-      <c r="F100" s="1"/>
-      <c r="G100" s="1"/>
-      <c r="H100" s="1"/>
-      <c r="I100" s="1"/>
-      <c r="J100" s="1"/>
-      <c r="K100" s="1"/>
-      <c r="L100" s="1"/>
-      <c r="M100" s="1"/>
+      <c r="B100" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="E100" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="F100" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H100" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I100" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="J100" s="8">
+        <v>3.105255156E9</v>
+      </c>
+      <c r="K100" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L100" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="M100" s="10" t="s">
+        <v>396</v>
+      </c>
       <c r="N100" s="1"/>
       <c r="O100" s="1"/>
       <c r="P100" s="1"/>
@@ -14457,18 +14784,42 @@
     </row>
     <row r="101" ht="14.25" customHeight="1">
       <c r="A101" s="1"/>
-      <c r="B101" s="1"/>
-      <c r="C101" s="1"/>
-      <c r="D101" s="1"/>
-      <c r="E101" s="1"/>
-      <c r="F101" s="1"/>
-      <c r="G101" s="1"/>
-      <c r="H101" s="1"/>
-      <c r="I101" s="1"/>
-      <c r="J101" s="1"/>
-      <c r="K101" s="1"/>
-      <c r="L101" s="1"/>
-      <c r="M101" s="1"/>
+      <c r="B101" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="C101" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="D101" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="E101" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G101" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I101" s="8" t="s">
+        <v>398</v>
+      </c>
+      <c r="J101" s="8">
+        <v>3.052047405E9</v>
+      </c>
+      <c r="K101" s="8">
+        <v>6.043221126E9</v>
+      </c>
+      <c r="L101" s="10" t="s">
+        <v>399</v>
+      </c>
+      <c r="M101" s="8" t="s">
+        <v>30</v>
+      </c>
       <c r="N101" s="1"/>
       <c r="O101" s="1"/>
       <c r="P101" s="1"/>
@@ -38777,12 +39128,23 @@
     <hyperlink r:id="rId24" ref="M90"/>
     <hyperlink r:id="rId25" ref="L91"/>
     <hyperlink r:id="rId26" ref="M91"/>
+    <hyperlink r:id="rId27" ref="M93"/>
+    <hyperlink r:id="rId28" ref="M94"/>
+    <hyperlink r:id="rId29" ref="M95"/>
+    <hyperlink r:id="rId30" ref="L96"/>
+    <hyperlink r:id="rId31" ref="M96"/>
+    <hyperlink r:id="rId32" ref="L97"/>
+    <hyperlink r:id="rId33" ref="M97"/>
+    <hyperlink r:id="rId34" ref="L98"/>
+    <hyperlink r:id="rId35" ref="M99"/>
+    <hyperlink r:id="rId36" ref="M100"/>
+    <hyperlink r:id="rId37" ref="L101"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId27"/>
-  <legacyDrawing r:id="rId28"/>
+  <drawing r:id="rId38"/>
+  <legacyDrawing r:id="rId39"/>
 </worksheet>
 </file>
 
@@ -38807,10 +39169,10 @@
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
-        <v>358</v>
+        <v>400</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>359</v>
+        <v>401</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -38819,10 +39181,10 @@
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
-        <v>360</v>
+        <v>402</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>361</v>
+        <v>403</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -38831,10 +39193,10 @@
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>360</v>
+        <v>402</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>362</v>
+        <v>404</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>

</xml_diff>